<commit_message>
fixed a bug related to the adjustment of test value error calculation relocated added adaptation and fixed test data calculation
</commit_message>
<xml_diff>
--- a/test_data.xlsx
+++ b/test_data.xlsx
@@ -110,7 +110,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -121,6 +121,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -267,7 +271,7 @@
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="3" t="n">
         <v>3</v>
       </c>
     </row>
@@ -278,7 +282,7 @@
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -289,7 +293,7 @@
       <c r="B4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="3" t="n">
         <v>3</v>
       </c>
     </row>
@@ -300,7 +304,7 @@
       <c r="B5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="3" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>